<commit_message>
Phase 5 Sprint 2 - P1 endpoints (SIM-355/356/357/358/359): /games/{date}, /simulate, /with_override, /plays, /state + persistence (Alembic 0014, DuckDB v9); suite 1661 green
</commit_message>
<xml_diff>
--- a/backlog.xlsx
+++ b/backlog.xlsx
@@ -15068,1664 +15068,1664 @@
       </c>
     </row>
     <row r="152">
-      <c r="A152" t="inlineStr">
+      <c r="A152" s="46" t="inlineStr">
         <is>
           <t>SIM-350</t>
         </is>
       </c>
-      <c r="B152" t="inlineStr">
+      <c r="B152" s="46" t="inlineStr">
         <is>
           <t>API response-serialization contract — Pydantic models + array-safe JSON for GameSimSummary/WinProbability/snapshots/PMFs/EdgeReport</t>
         </is>
       </c>
-      <c r="C152" t="inlineStr">
+      <c r="C152" s="46" t="inlineStr">
         <is>
           <t>Phase 5 — Backend API</t>
         </is>
       </c>
-      <c r="D152" t="inlineStr">
+      <c r="D152" s="46" t="inlineStr">
         <is>
           <t>Spec</t>
         </is>
       </c>
-      <c r="E152" t="inlineStr">
+      <c r="E152" s="46" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="F152" t="inlineStr">
+      <c r="F152" s="46" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="G152" t="inlineStr">
+      <c r="G152" s="46" t="inlineStr">
         <is>
           <t>Backend Developer · UX Designer</t>
         </is>
       </c>
-      <c r="H152" t="inlineStr">
+      <c r="H152" s="46" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
       </c>
-      <c r="I152" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J152" t="inlineStr">
+      <c r="I152" s="46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J152" s="46" t="inlineStr">
         <is>
           <t>Numpy-bearing output dataclasses had no JSON contract.</t>
         </is>
       </c>
-      <c r="K152" t="inlineStr">
+      <c r="K152" s="46" t="inlineStr">
         <is>
           <t>api/serialization.py + api/schemas.py; model_dump_json round-trips with no numpy leak.</t>
         </is>
       </c>
-      <c r="L152" t="inlineStr"/>
-      <c r="M152" t="inlineStr">
+      <c r="L152" s="46" t="inlineStr"/>
+      <c r="M152" s="46" t="inlineStr">
         <is>
           <t>Closed 2026-05-24 (Sprint 1). 21 tests.</t>
         </is>
       </c>
     </row>
     <row r="153">
-      <c r="A153" t="inlineStr">
+      <c r="A153" s="46" t="inlineStr">
         <is>
           <t>SIM-351</t>
         </is>
       </c>
-      <c r="B153" t="inlineStr">
+      <c r="B153" s="46" t="inlineStr">
         <is>
           <t>Auth + rate-limit + CORS baseline</t>
         </is>
       </c>
-      <c r="C153" t="inlineStr">
+      <c r="C153" s="46" t="inlineStr">
         <is>
           <t>Phase 5 — Backend API</t>
         </is>
       </c>
-      <c r="D153" t="inlineStr">
+      <c r="D153" s="46" t="inlineStr">
         <is>
           <t>Feature</t>
         </is>
       </c>
-      <c r="E153" t="inlineStr">
+      <c r="E153" s="46" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="F153" t="inlineStr">
+      <c r="F153" s="46" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="G153" t="inlineStr">
+      <c r="G153" s="46" t="inlineStr">
         <is>
           <t>Backend Developer · QA/DevOps</t>
         </is>
       </c>
-      <c r="H153" t="inlineStr">
+      <c r="H153" s="46" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
       </c>
-      <c r="I153" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J153" t="inlineStr">
+      <c r="I153" s="46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J153" s="46" t="inlineStr">
         <is>
           <t>No auth/rate-limit anywhere; CORS was ['*'].</t>
         </is>
       </c>
-      <c r="K153" t="inlineStr">
+      <c r="K153" s="46" t="inlineStr">
         <is>
           <t>api/auth.py: API-key dep + stdlib rate limiter + env CORS.</t>
         </is>
       </c>
-      <c r="L153" t="inlineStr"/>
-      <c r="M153" t="inlineStr">
+      <c r="L153" s="46" t="inlineStr"/>
+      <c r="M153" s="46" t="inlineStr">
         <is>
           <t>Closed 2026-05-24 (Sprint 1). 9 tests.</t>
         </is>
       </c>
     </row>
     <row r="154">
-      <c r="A154" t="inlineStr">
+      <c r="A154" s="46" t="inlineStr">
         <is>
           <t>SIM-352</t>
         </is>
       </c>
-      <c r="B154" t="inlineStr">
+      <c r="B154" s="46" t="inlineStr">
         <is>
           <t>Production DB-backed machine_factory for BatchRunner (real sims over PlayPoolSampler + SIM-333 tiles)</t>
         </is>
       </c>
-      <c r="C154" t="inlineStr">
+      <c r="C154" s="46" t="inlineStr">
         <is>
           <t>Phase 5 — Backend API</t>
         </is>
       </c>
-      <c r="D154" t="inlineStr">
+      <c r="D154" s="46" t="inlineStr">
         <is>
           <t>Feature</t>
         </is>
       </c>
-      <c r="E154" t="inlineStr">
+      <c r="E154" s="46" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="F154" t="inlineStr">
+      <c r="F154" s="46" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="G154" t="inlineStr">
+      <c r="G154" s="46" t="inlineStr">
         <is>
           <t>Backend Developer · Performance Engineer · ML Engineer</t>
         </is>
       </c>
-      <c r="H154" t="inlineStr">
+      <c r="H154" s="46" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
       </c>
-      <c r="I154" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J154" t="inlineStr">
+      <c r="I154" s="46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J154" s="46" t="inlineStr">
         <is>
           <t>Only the no-DB rng factory existed; /simulate couldn't run a real game.</t>
         </is>
       </c>
-      <c r="K154" t="inlineStr">
+      <c r="K154" s="46" t="inlineStr">
         <is>
           <t>simulation/production_factory.py; injectable builders for no-DB tests.</t>
         </is>
       </c>
-      <c r="L154" t="inlineStr"/>
-      <c r="M154" t="inlineStr">
+      <c r="L154" s="46" t="inlineStr"/>
+      <c r="M154" s="46" t="inlineStr">
         <is>
           <t>Closed 2026-05-24 (Sprint 1). 13 tests. Live-DB SLA acceptance → SIM-372.</t>
         </is>
       </c>
     </row>
     <row r="155">
-      <c r="A155" t="inlineStr">
+      <c r="A155" s="46" t="inlineStr">
         <is>
           <t>SIM-353</t>
         </is>
       </c>
-      <c r="B155" t="inlineStr">
+      <c r="B155" s="46" t="inlineStr">
         <is>
           <t>Runtime lineup/substitution resolver: Postgres raw.game_lineups → GameState (the SIM-338 gap)</t>
         </is>
       </c>
-      <c r="C155" t="inlineStr">
+      <c r="C155" s="46" t="inlineStr">
         <is>
           <t>Phase 5 — Backend API</t>
         </is>
       </c>
-      <c r="D155" t="inlineStr">
+      <c r="D155" s="46" t="inlineStr">
         <is>
           <t>Feature</t>
         </is>
       </c>
-      <c r="E155" t="inlineStr">
+      <c r="E155" s="46" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="F155" t="inlineStr">
+      <c r="F155" s="46" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="G155" t="inlineStr">
+      <c r="G155" s="46" t="inlineStr">
         <is>
           <t>Data Engineer · Backend Developer</t>
         </is>
       </c>
-      <c r="H155" t="inlineStr">
+      <c r="H155" s="46" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
       </c>
-      <c r="I155" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J155" t="inlineStr">
+      <c r="I155" s="46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J155" s="46" t="inlineStr">
         <is>
           <t>No runtime read path from lineup stores to GameState.</t>
         </is>
       </c>
-      <c r="K155" t="inlineStr">
+      <c r="K155" s="46" t="inlineStr">
         <is>
           <t>simulation/lineup_resolver.py; subs by sequence + as_of_at_bat.</t>
         </is>
       </c>
-      <c r="L155" t="inlineStr"/>
-      <c r="M155" t="inlineStr">
+      <c r="L155" s="46" t="inlineStr"/>
+      <c r="M155" s="46" t="inlineStr">
         <is>
           <t>Closed 2026-05-24 (Sprint 1). 24 tests. raw.game_lineups already in migration 0001.</t>
         </is>
       </c>
     </row>
     <row r="156">
-      <c r="A156" t="inlineStr">
+      <c r="A156" s="46" t="inlineStr">
         <is>
           <t>SIM-354</t>
         </is>
       </c>
-      <c r="B156" t="inlineStr">
+      <c r="B156" s="46" t="inlineStr">
         <is>
           <t>API skeleton — mount ws_router/odds_router/live pipeline into api/main.py</t>
         </is>
       </c>
-      <c r="C156" t="inlineStr">
+      <c r="C156" s="46" t="inlineStr">
         <is>
           <t>Phase 5 — Backend API</t>
         </is>
       </c>
-      <c r="D156" t="inlineStr">
+      <c r="D156" s="46" t="inlineStr">
         <is>
           <t>Gap</t>
         </is>
       </c>
-      <c r="E156" t="inlineStr">
+      <c r="E156" s="46" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="F156" t="inlineStr">
+      <c r="F156" s="46" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="G156" t="inlineStr">
+      <c r="G156" s="46" t="inlineStr">
         <is>
           <t>Backend Developer · Data Engineer</t>
         </is>
       </c>
-      <c r="H156" t="inlineStr">
+      <c r="H156" s="46" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
       </c>
-      <c r="I156" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J156" t="inlineStr">
+      <c r="I156" s="46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J156" s="46" t="inlineStr">
         <is>
           <t>Built routers/pipeline never mounted into the app.</t>
         </is>
       </c>
-      <c r="K156" t="inlineStr">
+      <c r="K156" s="46" t="inlineStr">
         <is>
           <t>api/main.py mounts routers; pipeline gated by LIVE_PIPELINE_ENABLED.</t>
         </is>
       </c>
-      <c r="L156" t="inlineStr"/>
-      <c r="M156" t="inlineStr">
+      <c r="L156" s="46" t="inlineStr"/>
+      <c r="M156" s="46" t="inlineStr">
         <is>
           <t>Closed 2026-05-24 (Sprint 1). 11 tests.</t>
         </is>
       </c>
     </row>
     <row r="157">
-      <c r="A157" t="inlineStr">
+      <c r="A157" s="46" t="inlineStr">
         <is>
           <t>SIM-355</t>
         </is>
       </c>
-      <c r="B157" t="inlineStr">
+      <c r="B157" s="46" t="inlineStr">
         <is>
           <t>GET /api/games/{date} + GET /{game_pk}/simulate (100-iteration runner → GameSimSummary)</t>
         </is>
       </c>
-      <c r="C157" t="inlineStr">
+      <c r="C157" s="46" t="inlineStr">
         <is>
           <t>Phase 5 — Backend API</t>
         </is>
       </c>
-      <c r="D157" t="inlineStr">
+      <c r="D157" s="46" t="inlineStr">
         <is>
           <t>Feature</t>
         </is>
       </c>
-      <c r="E157" t="inlineStr">
+      <c r="E157" s="46" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="F157" t="inlineStr">
+      <c r="F157" s="46" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="G157" t="inlineStr">
+      <c r="G157" s="46" t="inlineStr">
         <is>
           <t>Backend Developer</t>
         </is>
       </c>
-      <c r="H157" t="inlineStr">
+      <c r="H157" s="46" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="I157" s="46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J157" s="46" t="inlineStr">
+        <is>
+          <t>The core endpoints.</t>
+        </is>
+      </c>
+      <c r="K157" s="46" t="inlineStr"/>
+      <c r="L157" s="46" t="inlineStr"/>
+      <c r="M157" s="46" t="inlineStr">
+        <is>
+          <t>SIM-350, SIM-352, SIM-353 | Closed 2026-05-24 (Phase 5 Sprint 2).</t>
+        </is>
+      </c>
+      <c r="N157" s="46" t="inlineStr"/>
+    </row>
+    <row r="158">
+      <c r="A158" s="46" t="inlineStr">
+        <is>
+          <t>SIM-356</t>
+        </is>
+      </c>
+      <c r="B158" s="46" t="inlineStr">
+        <is>
+          <t>Sim-result + pitch-snapshot persistence (Alembic 0014 / DuckDB v8) backing /state + /plays</t>
+        </is>
+      </c>
+      <c r="C158" s="46" t="inlineStr">
+        <is>
+          <t>Phase 5 — Backend API</t>
+        </is>
+      </c>
+      <c r="D158" s="46" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E158" s="46" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F158" s="46" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="G158" s="46" t="inlineStr">
+        <is>
+          <t>Data Engineer</t>
+        </is>
+      </c>
+      <c r="H158" s="46" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="I158" s="46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J158" s="46" t="inlineStr">
+        <is>
+          <t>Only an ephemeral Redis/JSONB blob today.</t>
+        </is>
+      </c>
+      <c r="K158" s="46" t="inlineStr"/>
+      <c r="L158" s="46" t="inlineStr"/>
+      <c r="M158" s="46" t="inlineStr">
+        <is>
+          <t>SIM-350 | Closed 2026-05-24 (Phase 5 Sprint 2).</t>
+        </is>
+      </c>
+      <c r="N158" s="46" t="inlineStr"/>
+    </row>
+    <row r="159">
+      <c r="A159" s="46" t="inlineStr">
+        <is>
+          <t>SIM-357</t>
+        </is>
+      </c>
+      <c r="B159" s="46" t="inlineStr">
+        <is>
+          <t>GET /{game_pk}/plays + GET /{game_pk}/state/{at_bat}/{pitch} (from persisted snapshots)</t>
+        </is>
+      </c>
+      <c r="C159" s="46" t="inlineStr">
+        <is>
+          <t>Phase 5 — Backend API</t>
+        </is>
+      </c>
+      <c r="D159" s="46" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E159" s="46" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F159" s="46" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="G159" s="46" t="inlineStr">
+        <is>
+          <t>Backend Developer</t>
+        </is>
+      </c>
+      <c r="H159" s="46" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="I159" s="46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J159" s="46" t="inlineStr"/>
+      <c r="K159" s="46" t="inlineStr"/>
+      <c r="L159" s="46" t="inlineStr"/>
+      <c r="M159" s="46" t="inlineStr">
+        <is>
+          <t>SIM-356 | Closed 2026-05-24 (Phase 5 Sprint 2).</t>
+        </is>
+      </c>
+      <c r="N159" s="46" t="inlineStr"/>
+    </row>
+    <row r="160">
+      <c r="A160" s="46" t="inlineStr">
+        <is>
+          <t>SIM-358</t>
+        </is>
+      </c>
+      <c r="B160" s="46" t="inlineStr">
+        <is>
+          <t>POST /{game_pk}/simulate/with_override (roster-mod re-sim → OverrideDelta)</t>
+        </is>
+      </c>
+      <c r="C160" s="46" t="inlineStr">
+        <is>
+          <t>Phase 5 — Backend API</t>
+        </is>
+      </c>
+      <c r="D160" s="46" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E160" s="46" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F160" s="46" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="G160" s="46" t="inlineStr">
+        <is>
+          <t>Backend Developer</t>
+        </is>
+      </c>
+      <c r="H160" s="46" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="I160" s="46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J160" s="46" t="inlineStr"/>
+      <c r="K160" s="46" t="inlineStr"/>
+      <c r="L160" s="46" t="inlineStr"/>
+      <c r="M160" s="46" t="inlineStr">
+        <is>
+          <t>SIM-355 | Closed 2026-05-24 (Phase 5 Sprint 2).</t>
+        </is>
+      </c>
+      <c r="N160" s="46" t="inlineStr"/>
+    </row>
+    <row r="161">
+      <c r="A161" s="46" t="inlineStr">
+        <is>
+          <t>SIM-359</t>
+        </is>
+      </c>
+      <c r="B161" s="46" t="inlineStr">
+        <is>
+          <t>Redis TTL wiring for the API (sim 60s / pool 5-min / odds 5-min)</t>
+        </is>
+      </c>
+      <c r="C161" s="46" t="inlineStr">
+        <is>
+          <t>Phase 5 — Backend API</t>
+        </is>
+      </c>
+      <c r="D161" s="46" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E161" s="46" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F161" s="46" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G161" s="46" t="inlineStr">
+        <is>
+          <t>Backend Developer</t>
+        </is>
+      </c>
+      <c r="H161" s="46" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="I161" s="46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J161" s="46" t="inlineStr">
+        <is>
+          <t>Constants exist; not wired to the API.</t>
+        </is>
+      </c>
+      <c r="K161" s="46" t="inlineStr"/>
+      <c r="L161" s="46" t="inlineStr"/>
+      <c r="M161" s="46" t="inlineStr">
+        <is>
+          <t>SIM-355 | Closed 2026-05-24 (Phase 5 Sprint 2).</t>
+        </is>
+      </c>
+      <c r="N161" s="46" t="inlineStr"/>
+    </row>
+    <row r="162">
+      <c r="A162" s="46" t="inlineStr">
+        <is>
+          <t>SIM-360</t>
+        </is>
+      </c>
+      <c r="B162" s="46" t="inlineStr">
+        <is>
+          <t>Persistent ProcessPool + shared-memory lifecycle for the long-lived API</t>
+        </is>
+      </c>
+      <c r="C162" s="46" t="inlineStr">
+        <is>
+          <t>Phase 5 — Backend API</t>
+        </is>
+      </c>
+      <c r="D162" s="46" t="inlineStr">
+        <is>
+          <t>Perf</t>
+        </is>
+      </c>
+      <c r="E162" s="46" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F162" s="46" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="G162" s="46" t="inlineStr">
+        <is>
+          <t>Performance Engineer</t>
+        </is>
+      </c>
+      <c r="H162" s="46" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="I157" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J157" t="inlineStr">
-        <is>
-          <t>The core endpoints.</t>
-        </is>
-      </c>
-      <c r="K157" t="inlineStr"/>
-      <c r="L157" t="inlineStr"/>
-      <c r="M157" t="inlineStr">
-        <is>
-          <t>SIM-350, SIM-352, SIM-353</t>
-        </is>
-      </c>
-      <c r="N157" t="inlineStr"/>
-    </row>
-    <row r="158">
-      <c r="A158" t="inlineStr">
-        <is>
-          <t>SIM-356</t>
-        </is>
-      </c>
-      <c r="B158" t="inlineStr">
-        <is>
-          <t>Sim-result + pitch-snapshot persistence (Alembic 0014 / DuckDB v8) backing /state + /plays</t>
-        </is>
-      </c>
-      <c r="C158" t="inlineStr">
+      <c r="I162" s="46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J162" s="46" t="inlineStr">
+        <is>
+          <t>Today a fresh pool + shm publish/unlink per request.</t>
+        </is>
+      </c>
+      <c r="K162" s="46" t="inlineStr"/>
+      <c r="L162" s="46" t="inlineStr"/>
+      <c r="M162" s="46" t="inlineStr">
+        <is>
+          <t>SIM-352</t>
+        </is>
+      </c>
+      <c r="N162" s="46" t="inlineStr"/>
+    </row>
+    <row r="163">
+      <c r="A163" s="46" t="inlineStr">
+        <is>
+          <t>SIM-361</t>
+        </is>
+      </c>
+      <c r="B163" s="46" t="inlineStr">
+        <is>
+          <t>CalibrationReport JSON persistence + API-startup load + CalibrationMap wiring; build all 11 engines</t>
+        </is>
+      </c>
+      <c r="C163" s="46" t="inlineStr">
         <is>
           <t>Phase 5 — Backend API</t>
         </is>
       </c>
-      <c r="D158" t="inlineStr">
+      <c r="D163" s="46" t="inlineStr">
         <is>
           <t>Feature</t>
         </is>
       </c>
-      <c r="E158" t="inlineStr">
+      <c r="E163" s="46" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="F158" t="inlineStr">
+      <c r="F163" s="46" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="G158" t="inlineStr">
-        <is>
-          <t>Data Engineer</t>
-        </is>
-      </c>
-      <c r="H158" t="inlineStr">
+      <c r="G163" s="46" t="inlineStr">
+        <is>
+          <t>ML Engineer</t>
+        </is>
+      </c>
+      <c r="H163" s="46" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="I158" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J158" t="inlineStr">
-        <is>
-          <t>Only an ephemeral Redis/JSONB blob today.</t>
-        </is>
-      </c>
-      <c r="K158" t="inlineStr"/>
-      <c r="L158" t="inlineStr"/>
-      <c r="M158" t="inlineStr">
+      <c r="I163" s="46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J163" s="46" t="inlineStr">
+        <is>
+          <t>Only the pitcher engine builds at startup today.</t>
+        </is>
+      </c>
+      <c r="K163" s="46" t="inlineStr"/>
+      <c r="L163" s="46" t="inlineStr"/>
+      <c r="M163" s="46" t="inlineStr"/>
+      <c r="N163" s="46" t="inlineStr"/>
+    </row>
+    <row r="164">
+      <c r="A164" s="46" t="inlineStr">
+        <is>
+          <t>SIM-362</t>
+        </is>
+      </c>
+      <c r="B164" s="46" t="inlineStr">
+        <is>
+          <t>Per-inning linescore + team R/H/E tracking in the loop</t>
+        </is>
+      </c>
+      <c r="C164" s="46" t="inlineStr">
+        <is>
+          <t>Phase 5 — Loop Outputs</t>
+        </is>
+      </c>
+      <c r="D164" s="46" t="inlineStr">
+        <is>
+          <t>Gap</t>
+        </is>
+      </c>
+      <c r="E164" s="46" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F164" s="46" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G164" s="46" t="inlineStr">
+        <is>
+          <t>Backend Developer · Baseball Analyst</t>
+        </is>
+      </c>
+      <c r="H164" s="46" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I164" s="46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J164" s="46" t="inlineStr">
+        <is>
+          <t>Only cumulative score exists; LinescoreGraphic unservable.</t>
+        </is>
+      </c>
+      <c r="K164" s="46" t="inlineStr"/>
+      <c r="L164" s="46" t="inlineStr"/>
+      <c r="M164" s="46" t="inlineStr"/>
+      <c r="N164" s="46" t="inlineStr"/>
+    </row>
+    <row r="165">
+      <c r="A165" s="46" t="inlineStr">
+        <is>
+          <t>SIM-363</t>
+        </is>
+      </c>
+      <c r="B165" s="46" t="inlineStr">
+        <is>
+          <t>Per-position fielder tracking → populate FieldSnapshot's 9 defensive slots</t>
+        </is>
+      </c>
+      <c r="C165" s="46" t="inlineStr">
+        <is>
+          <t>Phase 5 — Loop Outputs</t>
+        </is>
+      </c>
+      <c r="D165" s="46" t="inlineStr">
+        <is>
+          <t>Gap</t>
+        </is>
+      </c>
+      <c r="E165" s="46" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F165" s="46" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="G165" s="46" t="inlineStr">
+        <is>
+          <t>Backend Developer · ML Engineer</t>
+        </is>
+      </c>
+      <c r="H165" s="46" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I165" s="46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J165" s="46" t="inlineStr">
+        <is>
+          <t>FieldSnapshot slots empty today.</t>
+        </is>
+      </c>
+      <c r="K165" s="46" t="inlineStr"/>
+      <c r="L165" s="46" t="inlineStr"/>
+      <c r="M165" s="46" t="inlineStr">
+        <is>
+          <t>SIM-353</t>
+        </is>
+      </c>
+      <c r="N165" s="46" t="inlineStr"/>
+    </row>
+    <row r="166">
+      <c r="A166" s="46" t="inlineStr">
+        <is>
+          <t>SIM-364</t>
+        </is>
+      </c>
+      <c r="B166" s="46" t="inlineStr">
+        <is>
+          <t>Winning / losing / save pitcher attribution</t>
+        </is>
+      </c>
+      <c r="C166" s="46" t="inlineStr">
+        <is>
+          <t>Phase 5 — Loop Outputs</t>
+        </is>
+      </c>
+      <c r="D166" s="46" t="inlineStr">
+        <is>
+          <t>Gap</t>
+        </is>
+      </c>
+      <c r="E166" s="46" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F166" s="46" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="G166" s="46" t="inlineStr">
+        <is>
+          <t>Baseball Analyst · Backend Developer</t>
+        </is>
+      </c>
+      <c r="H166" s="46" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I166" s="46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J166" s="46" t="inlineStr">
+        <is>
+          <t>Required by the Completed game card; absent today.</t>
+        </is>
+      </c>
+      <c r="K166" s="46" t="inlineStr"/>
+      <c r="L166" s="46" t="inlineStr"/>
+      <c r="M166" s="46" t="inlineStr">
+        <is>
+          <t>SIM-362</t>
+        </is>
+      </c>
+      <c r="N166" s="46" t="inlineStr"/>
+    </row>
+    <row r="167">
+      <c r="A167" s="46" t="inlineStr">
+        <is>
+          <t>SIM-365</t>
+        </is>
+      </c>
+      <c r="B167" s="46" t="inlineStr">
+        <is>
+          <t>Extend PlayerStatLine (2B/3B/R/SB; pitcher hits/runs-allowed) + fix SIM-329 prop-TB lower bound</t>
+        </is>
+      </c>
+      <c r="C167" s="46" t="inlineStr">
+        <is>
+          <t>Phase 5 — Loop Outputs</t>
+        </is>
+      </c>
+      <c r="D167" s="46" t="inlineStr">
+        <is>
+          <t>Improvement</t>
+        </is>
+      </c>
+      <c r="E167" s="46" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F167" s="46" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="G167" s="46" t="inlineStr">
+        <is>
+          <t>Baseball Analyst · Backend Developer</t>
+        </is>
+      </c>
+      <c r="H167" s="46" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I167" s="46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J167" s="46" t="inlineStr">
+        <is>
+          <t>prop TB is a lower bound (h+3·hr) until 2B/3B tracked.</t>
+        </is>
+      </c>
+      <c r="K167" s="46" t="inlineStr"/>
+      <c r="L167" s="46" t="inlineStr"/>
+      <c r="M167" s="46" t="inlineStr"/>
+      <c r="N167" s="46" t="inlineStr"/>
+    </row>
+    <row r="168">
+      <c r="A168" s="46" t="inlineStr">
+        <is>
+          <t>SIM-366</t>
+        </is>
+      </c>
+      <c r="B168" s="46" t="inlineStr">
+        <is>
+          <t>Per-player 100-iteration boxscore-average API shape (PropDistributionSet means)</t>
+        </is>
+      </c>
+      <c r="C168" s="46" t="inlineStr">
+        <is>
+          <t>Phase 5 — Backend API</t>
+        </is>
+      </c>
+      <c r="D168" s="46" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E168" s="46" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F168" s="46" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G168" s="46" t="inlineStr">
+        <is>
+          <t>Backend Developer · UX Designer</t>
+        </is>
+      </c>
+      <c r="H168" s="46" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I168" s="46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J168" s="46" t="inlineStr"/>
+      <c r="K168" s="46" t="inlineStr"/>
+      <c r="L168" s="46" t="inlineStr"/>
+      <c r="M168" s="46" t="inlineStr">
         <is>
           <t>SIM-350</t>
         </is>
       </c>
-      <c r="N158" t="inlineStr"/>
-    </row>
-    <row r="159">
-      <c r="A159" t="inlineStr">
-        <is>
-          <t>SIM-357</t>
-        </is>
-      </c>
-      <c r="B159" t="inlineStr">
-        <is>
-          <t>GET /{game_pk}/plays + GET /{game_pk}/state/{at_bat}/{pitch} (from persisted snapshots)</t>
-        </is>
-      </c>
-      <c r="C159" t="inlineStr">
-        <is>
-          <t>Phase 5 — Backend API</t>
-        </is>
-      </c>
-      <c r="D159" t="inlineStr">
+      <c r="N168" s="46" t="inlineStr"/>
+    </row>
+    <row r="169">
+      <c r="A169" s="46" t="inlineStr">
+        <is>
+          <t>SIM-367</t>
+        </is>
+      </c>
+      <c r="B169" s="46" t="inlineStr">
+        <is>
+          <t>Run-line / spread EdgeReport from raw score-margin arrays</t>
+        </is>
+      </c>
+      <c r="C169" s="46" t="inlineStr">
+        <is>
+          <t>Phase 5 — Betting</t>
+        </is>
+      </c>
+      <c r="D169" s="46" t="inlineStr">
+        <is>
+          <t>Gap</t>
+        </is>
+      </c>
+      <c r="E169" s="46" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F169" s="46" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G169" s="46" t="inlineStr">
+        <is>
+          <t>Betting Analyst · ML Engineer</t>
+        </is>
+      </c>
+      <c r="H169" s="46" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I169" s="46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J169" s="46" t="inlineStr">
+        <is>
+          <t>Only ML/total/prop edge exist.</t>
+        </is>
+      </c>
+      <c r="K169" s="46" t="inlineStr"/>
+      <c r="L169" s="46" t="inlineStr"/>
+      <c r="M169" s="46" t="inlineStr"/>
+      <c r="N169" s="46" t="inlineStr"/>
+    </row>
+    <row r="170">
+      <c r="A170" s="46" t="inlineStr">
+        <is>
+          <t>SIM-368</t>
+        </is>
+      </c>
+      <c r="B170" s="46" t="inlineStr">
+        <is>
+          <t>CLV / line-movement time-series surface (opening→closing)</t>
+        </is>
+      </c>
+      <c r="C170" s="46" t="inlineStr">
+        <is>
+          <t>Phase 5 — Betting</t>
+        </is>
+      </c>
+      <c r="D170" s="46" t="inlineStr">
+        <is>
+          <t>Gap</t>
+        </is>
+      </c>
+      <c r="E170" s="46" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F170" s="46" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="G170" s="46" t="inlineStr">
+        <is>
+          <t>Betting Analyst · Data Engineer</t>
+        </is>
+      </c>
+      <c r="H170" s="46" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I170" s="46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J170" s="46" t="inlineStr">
+        <is>
+          <t>CLV is a single entry-vs-close snapshot today.</t>
+        </is>
+      </c>
+      <c r="K170" s="46" t="inlineStr"/>
+      <c r="L170" s="46" t="inlineStr"/>
+      <c r="M170" s="46" t="inlineStr">
+        <is>
+          <t>SIM-370</t>
+        </is>
+      </c>
+      <c r="N170" s="46" t="inlineStr"/>
+    </row>
+    <row r="171">
+      <c r="A171" s="46" t="inlineStr">
+        <is>
+          <t>SIM-369</t>
+        </is>
+      </c>
+      <c r="B171" s="46" t="inlineStr">
+        <is>
+          <t>Bet-signal / +EV recommendation endpoint contract</t>
+        </is>
+      </c>
+      <c r="C171" s="46" t="inlineStr">
+        <is>
+          <t>Phase 5 — Betting</t>
+        </is>
+      </c>
+      <c r="D171" s="46" t="inlineStr">
         <is>
           <t>Feature</t>
         </is>
       </c>
-      <c r="E159" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="F159" t="inlineStr">
+      <c r="E171" s="46" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F171" s="46" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="G159" t="inlineStr">
+      <c r="G171" s="46" t="inlineStr">
+        <is>
+          <t>Betting Analyst</t>
+        </is>
+      </c>
+      <c r="H171" s="46" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I171" s="46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J171" s="46" t="inlineStr">
+        <is>
+          <t>Aggregate EdgeReports into a fireable signal.</t>
+        </is>
+      </c>
+      <c r="K171" s="46" t="inlineStr"/>
+      <c r="L171" s="46" t="inlineStr"/>
+      <c r="M171" s="46" t="inlineStr">
+        <is>
+          <t>SIM-367</t>
+        </is>
+      </c>
+      <c r="N171" s="46" t="inlineStr"/>
+    </row>
+    <row r="172">
+      <c r="A172" s="46" t="inlineStr">
+        <is>
+          <t>SIM-370</t>
+        </is>
+      </c>
+      <c r="B172" s="46" t="inlineStr">
+        <is>
+          <t>Real odds/prop provider swap behind MockOddsAPI</t>
+        </is>
+      </c>
+      <c r="C172" s="46" t="inlineStr">
+        <is>
+          <t>Phase 5 — Betting</t>
+        </is>
+      </c>
+      <c r="D172" s="46" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E172" s="46" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F172" s="46" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="G172" s="46" t="inlineStr">
+        <is>
+          <t>Data Engineer · Betting Analyst</t>
+        </is>
+      </c>
+      <c r="H172" s="46" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I172" s="46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J172" s="46" t="inlineStr">
+        <is>
+          <t>Multi-book, sharp flag; cadence wired by SIM-340.</t>
+        </is>
+      </c>
+      <c r="K172" s="46" t="inlineStr"/>
+      <c r="L172" s="46" t="inlineStr"/>
+      <c r="M172" s="46" t="inlineStr"/>
+      <c r="N172" s="46" t="inlineStr"/>
+    </row>
+    <row r="173">
+      <c r="A173" s="46" t="inlineStr">
+        <is>
+          <t>SIM-371</t>
+        </is>
+      </c>
+      <c r="B173" s="46" t="inlineStr">
+        <is>
+          <t>API integration + WebSocket + historical-replay E2E suite</t>
+        </is>
+      </c>
+      <c r="C173" s="46" t="inlineStr">
+        <is>
+          <t>Phase 5 — Testing</t>
+        </is>
+      </c>
+      <c r="D173" s="46" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="E173" s="46" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F173" s="46" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G173" s="46" t="inlineStr">
+        <is>
+          <t>QA/DevOps · Baseball Analyst</t>
+        </is>
+      </c>
+      <c r="H173" s="46" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I173" s="46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J173" s="46" t="inlineStr">
+        <is>
+          <t>api/websocket/ is an empty placeholder.</t>
+        </is>
+      </c>
+      <c r="K173" s="46" t="inlineStr"/>
+      <c r="L173" s="46" t="inlineStr"/>
+      <c r="M173" s="46" t="inlineStr">
+        <is>
+          <t>SIM-355</t>
+        </is>
+      </c>
+      <c r="N173" s="46" t="inlineStr"/>
+    </row>
+    <row r="174">
+      <c r="A174" s="46" t="inlineStr">
+        <is>
+          <t>SIM-372</t>
+        </is>
+      </c>
+      <c r="B174" s="46" t="inlineStr">
+        <is>
+          <t>End-to-end /simulate latency perf gate (2s/30s SLA)</t>
+        </is>
+      </c>
+      <c r="C174" s="46" t="inlineStr">
+        <is>
+          <t>Phase 5 — Testing</t>
+        </is>
+      </c>
+      <c r="D174" s="46" t="inlineStr">
+        <is>
+          <t>Perf</t>
+        </is>
+      </c>
+      <c r="E174" s="46" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F174" s="46" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="G174" s="46" t="inlineStr">
+        <is>
+          <t>Performance Engineer</t>
+        </is>
+      </c>
+      <c r="H174" s="46" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I174" s="46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J174" s="46" t="inlineStr">
+        <is>
+          <t>Current bench skips the request path.</t>
+        </is>
+      </c>
+      <c r="K174" s="46" t="inlineStr"/>
+      <c r="L174" s="46" t="inlineStr"/>
+      <c r="M174" s="46" t="inlineStr">
+        <is>
+          <t>SIM-352</t>
+        </is>
+      </c>
+      <c r="N174" s="46" t="inlineStr"/>
+    </row>
+    <row r="175">
+      <c r="A175" s="46" t="inlineStr">
+        <is>
+          <t>SIM-373</t>
+        </is>
+      </c>
+      <c r="B175" s="46" t="inlineStr">
+        <is>
+          <t>nginx reverse proxy w/ WebSocket upgrade + dev/staging/prod env configs</t>
+        </is>
+      </c>
+      <c r="C175" s="46" t="inlineStr">
+        <is>
+          <t>Phase 5 — Infra</t>
+        </is>
+      </c>
+      <c r="D175" s="46" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="E175" s="46" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="F175" s="46" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="G175" s="46" t="inlineStr">
+        <is>
+          <t>QA/DevOps</t>
+        </is>
+      </c>
+      <c r="H175" s="46" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I175" s="46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J175" s="46" t="inlineStr"/>
+      <c r="K175" s="46" t="inlineStr"/>
+      <c r="L175" s="46" t="inlineStr"/>
+      <c r="M175" s="46" t="inlineStr">
+        <is>
+          <t>SIM-354</t>
+        </is>
+      </c>
+      <c r="N175" s="46" t="inlineStr"/>
+    </row>
+    <row r="176">
+      <c r="A176" s="46" t="inlineStr">
+        <is>
+          <t>SIM-374</t>
+        </is>
+      </c>
+      <c r="B176" s="46" t="inlineStr">
+        <is>
+          <t>Prometheus + Grafana monitoring (sim latency, API p95, pipeline freshness)</t>
+        </is>
+      </c>
+      <c r="C176" s="46" t="inlineStr">
+        <is>
+          <t>Phase 5 — Infra</t>
+        </is>
+      </c>
+      <c r="D176" s="46" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="E176" s="46" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="F176" s="46" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="G176" s="46" t="inlineStr">
+        <is>
+          <t>QA/DevOps</t>
+        </is>
+      </c>
+      <c r="H176" s="46" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I176" s="46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J176" s="46" t="inlineStr"/>
+      <c r="K176" s="46" t="inlineStr"/>
+      <c r="L176" s="46" t="inlineStr"/>
+      <c r="M176" s="46" t="inlineStr">
+        <is>
+          <t>SIM-373</t>
+        </is>
+      </c>
+      <c r="N176" s="46" t="inlineStr"/>
+    </row>
+    <row r="177">
+      <c r="A177" s="46" t="inlineStr">
+        <is>
+          <t>SIM-375</t>
+        </is>
+      </c>
+      <c r="B177" s="46" t="inlineStr">
+        <is>
+          <t>Fix docker-compose.yml to mount ./simulation + remove the dead simulator/ package</t>
+        </is>
+      </c>
+      <c r="C177" s="46" t="inlineStr">
+        <is>
+          <t>Phase 5 — Infra</t>
+        </is>
+      </c>
+      <c r="D177" s="46" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="E177" s="46" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="F177" s="46" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G177" s="46" t="inlineStr">
+        <is>
+          <t>Data Engineer · QA/DevOps</t>
+        </is>
+      </c>
+      <c r="H177" s="46" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="I177" s="46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J177" s="46" t="inlineStr">
+        <is>
+          <t>Compose mounted the empty ./simulator stub.</t>
+        </is>
+      </c>
+      <c r="K177" s="46" t="inlineStr">
+        <is>
+          <t>compose mounts ./simulation; Dockerfile copies simulation/+betting/; simulator/ deleted.</t>
+        </is>
+      </c>
+      <c r="L177" s="46" t="inlineStr"/>
+      <c r="M177" s="46" t="inlineStr">
+        <is>
+          <t>Closed 2026-05-24 (Sprint 1).</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="46" t="inlineStr">
+        <is>
+          <t>SIM-376</t>
+        </is>
+      </c>
+      <c r="B178" s="46" t="inlineStr">
+        <is>
+          <t>Add api/ to the coverage gate (pyproject source + ci --cov=api)</t>
+        </is>
+      </c>
+      <c r="C178" s="46" t="inlineStr">
+        <is>
+          <t>Phase 5 — Infra</t>
+        </is>
+      </c>
+      <c r="D178" s="46" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="E178" s="46" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="F178" s="46" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G178" s="46" t="inlineStr">
+        <is>
+          <t>QA/DevOps</t>
+        </is>
+      </c>
+      <c r="H178" s="46" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="I178" s="46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J178" s="46" t="inlineStr">
+        <is>
+          <t>Only the Makefile measured api/ coverage.</t>
+        </is>
+      </c>
+      <c r="K178" s="46" t="inlineStr">
+        <is>
+          <t>pyproject source += api; ci --cov=api.</t>
+        </is>
+      </c>
+      <c r="L178" s="46" t="inlineStr"/>
+      <c r="M178" s="46" t="inlineStr">
+        <is>
+          <t>Closed 2026-05-24 (Sprint 1).</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="46" t="inlineStr">
+        <is>
+          <t>SIM-377</t>
+        </is>
+      </c>
+      <c r="B179" s="46" t="inlineStr">
+        <is>
+          <t>Fix/remove GameSpec._hit_rate (factory reads it but simulate_game has no **kwargs → TypeError)</t>
+        </is>
+      </c>
+      <c r="C179" s="46" t="inlineStr">
+        <is>
+          <t>Phase 5 — Infra</t>
+        </is>
+      </c>
+      <c r="D179" s="46" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="E179" s="46" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="F179" s="46" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G179" s="46" t="inlineStr">
         <is>
           <t>Backend Developer</t>
         </is>
       </c>
-      <c r="H159" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="I159" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J159" t="inlineStr"/>
-      <c r="K159" t="inlineStr"/>
-      <c r="L159" t="inlineStr"/>
-      <c r="M159" t="inlineStr">
-        <is>
-          <t>SIM-356</t>
-        </is>
-      </c>
-      <c r="N159" t="inlineStr"/>
-    </row>
-    <row r="160">
-      <c r="A160" t="inlineStr">
-        <is>
-          <t>SIM-358</t>
-        </is>
-      </c>
-      <c r="B160" t="inlineStr">
-        <is>
-          <t>POST /{game_pk}/simulate/with_override (roster-mod re-sim → OverrideDelta)</t>
-        </is>
-      </c>
-      <c r="C160" t="inlineStr">
-        <is>
-          <t>Phase 5 — Backend API</t>
-        </is>
-      </c>
-      <c r="D160" t="inlineStr">
-        <is>
-          <t>Feature</t>
-        </is>
-      </c>
-      <c r="E160" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="F160" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="G160" t="inlineStr">
-        <is>
-          <t>Backend Developer</t>
-        </is>
-      </c>
-      <c r="H160" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="I160" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J160" t="inlineStr"/>
-      <c r="K160" t="inlineStr"/>
-      <c r="L160" t="inlineStr"/>
-      <c r="M160" t="inlineStr">
-        <is>
-          <t>SIM-355</t>
-        </is>
-      </c>
-      <c r="N160" t="inlineStr"/>
-    </row>
-    <row r="161">
-      <c r="A161" t="inlineStr">
-        <is>
-          <t>SIM-359</t>
-        </is>
-      </c>
-      <c r="B161" t="inlineStr">
-        <is>
-          <t>Redis TTL wiring for the API (sim 60s / pool 5-min / odds 5-min)</t>
-        </is>
-      </c>
-      <c r="C161" t="inlineStr">
-        <is>
-          <t>Phase 5 — Backend API</t>
-        </is>
-      </c>
-      <c r="D161" t="inlineStr">
-        <is>
-          <t>Feature</t>
-        </is>
-      </c>
-      <c r="E161" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="F161" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="G161" t="inlineStr">
-        <is>
-          <t>Backend Developer</t>
-        </is>
-      </c>
-      <c r="H161" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="I161" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J161" t="inlineStr">
-        <is>
-          <t>Constants exist; not wired to the API.</t>
-        </is>
-      </c>
-      <c r="K161" t="inlineStr"/>
-      <c r="L161" t="inlineStr"/>
-      <c r="M161" t="inlineStr">
-        <is>
-          <t>SIM-355</t>
-        </is>
-      </c>
-      <c r="N161" t="inlineStr"/>
-    </row>
-    <row r="162">
-      <c r="A162" t="inlineStr">
-        <is>
-          <t>SIM-360</t>
-        </is>
-      </c>
-      <c r="B162" t="inlineStr">
-        <is>
-          <t>Persistent ProcessPool + shared-memory lifecycle for the long-lived API</t>
-        </is>
-      </c>
-      <c r="C162" t="inlineStr">
-        <is>
-          <t>Phase 5 — Backend API</t>
-        </is>
-      </c>
-      <c r="D162" t="inlineStr">
-        <is>
-          <t>Perf</t>
-        </is>
-      </c>
-      <c r="E162" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="F162" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="G162" t="inlineStr">
-        <is>
-          <t>Performance Engineer</t>
-        </is>
-      </c>
-      <c r="H162" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="I162" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J162" t="inlineStr">
-        <is>
-          <t>Today a fresh pool + shm publish/unlink per request.</t>
-        </is>
-      </c>
-      <c r="K162" t="inlineStr"/>
-      <c r="L162" t="inlineStr"/>
-      <c r="M162" t="inlineStr">
-        <is>
-          <t>SIM-352</t>
-        </is>
-      </c>
-      <c r="N162" t="inlineStr"/>
-    </row>
-    <row r="163">
-      <c r="A163" t="inlineStr">
-        <is>
-          <t>SIM-361</t>
-        </is>
-      </c>
-      <c r="B163" t="inlineStr">
-        <is>
-          <t>CalibrationReport JSON persistence + API-startup load + CalibrationMap wiring; build all 11 engines</t>
-        </is>
-      </c>
-      <c r="C163" t="inlineStr">
-        <is>
-          <t>Phase 5 — Backend API</t>
-        </is>
-      </c>
-      <c r="D163" t="inlineStr">
-        <is>
-          <t>Feature</t>
-        </is>
-      </c>
-      <c r="E163" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="F163" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="G163" t="inlineStr">
-        <is>
-          <t>ML Engineer</t>
-        </is>
-      </c>
-      <c r="H163" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="I163" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J163" t="inlineStr">
-        <is>
-          <t>Only the pitcher engine builds at startup today.</t>
-        </is>
-      </c>
-      <c r="K163" t="inlineStr"/>
-      <c r="L163" t="inlineStr"/>
-      <c r="M163" t="inlineStr"/>
-      <c r="N163" t="inlineStr"/>
-    </row>
-    <row r="164">
-      <c r="A164" t="inlineStr">
-        <is>
-          <t>SIM-362</t>
-        </is>
-      </c>
-      <c r="B164" t="inlineStr">
-        <is>
-          <t>Per-inning linescore + team R/H/E tracking in the loop</t>
-        </is>
-      </c>
-      <c r="C164" t="inlineStr">
-        <is>
-          <t>Phase 5 — Loop Outputs</t>
-        </is>
-      </c>
-      <c r="D164" t="inlineStr">
-        <is>
-          <t>Gap</t>
-        </is>
-      </c>
-      <c r="E164" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="F164" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="G164" t="inlineStr">
-        <is>
-          <t>Backend Developer · Baseball Analyst</t>
-        </is>
-      </c>
-      <c r="H164" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="I164" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J164" t="inlineStr">
-        <is>
-          <t>Only cumulative score exists; LinescoreGraphic unservable.</t>
-        </is>
-      </c>
-      <c r="K164" t="inlineStr"/>
-      <c r="L164" t="inlineStr"/>
-      <c r="M164" t="inlineStr"/>
-      <c r="N164" t="inlineStr"/>
-    </row>
-    <row r="165">
-      <c r="A165" t="inlineStr">
-        <is>
-          <t>SIM-363</t>
-        </is>
-      </c>
-      <c r="B165" t="inlineStr">
-        <is>
-          <t>Per-position fielder tracking → populate FieldSnapshot's 9 defensive slots</t>
-        </is>
-      </c>
-      <c r="C165" t="inlineStr">
-        <is>
-          <t>Phase 5 — Loop Outputs</t>
-        </is>
-      </c>
-      <c r="D165" t="inlineStr">
-        <is>
-          <t>Gap</t>
-        </is>
-      </c>
-      <c r="E165" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="F165" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="G165" t="inlineStr">
-        <is>
-          <t>Backend Developer · ML Engineer</t>
-        </is>
-      </c>
-      <c r="H165" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="I165" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J165" t="inlineStr">
-        <is>
-          <t>FieldSnapshot slots empty today.</t>
-        </is>
-      </c>
-      <c r="K165" t="inlineStr"/>
-      <c r="L165" t="inlineStr"/>
-      <c r="M165" t="inlineStr">
-        <is>
-          <t>SIM-353</t>
-        </is>
-      </c>
-      <c r="N165" t="inlineStr"/>
-    </row>
-    <row r="166">
-      <c r="A166" t="inlineStr">
-        <is>
-          <t>SIM-364</t>
-        </is>
-      </c>
-      <c r="B166" t="inlineStr">
-        <is>
-          <t>Winning / losing / save pitcher attribution</t>
-        </is>
-      </c>
-      <c r="C166" t="inlineStr">
-        <is>
-          <t>Phase 5 — Loop Outputs</t>
-        </is>
-      </c>
-      <c r="D166" t="inlineStr">
-        <is>
-          <t>Gap</t>
-        </is>
-      </c>
-      <c r="E166" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="F166" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="G166" t="inlineStr">
-        <is>
-          <t>Baseball Analyst · Backend Developer</t>
-        </is>
-      </c>
-      <c r="H166" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="I166" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J166" t="inlineStr">
-        <is>
-          <t>Required by the Completed game card; absent today.</t>
-        </is>
-      </c>
-      <c r="K166" t="inlineStr"/>
-      <c r="L166" t="inlineStr"/>
-      <c r="M166" t="inlineStr">
-        <is>
-          <t>SIM-362</t>
-        </is>
-      </c>
-      <c r="N166" t="inlineStr"/>
-    </row>
-    <row r="167">
-      <c r="A167" t="inlineStr">
-        <is>
-          <t>SIM-365</t>
-        </is>
-      </c>
-      <c r="B167" t="inlineStr">
-        <is>
-          <t>Extend PlayerStatLine (2B/3B/R/SB; pitcher hits/runs-allowed) + fix SIM-329 prop-TB lower bound</t>
-        </is>
-      </c>
-      <c r="C167" t="inlineStr">
-        <is>
-          <t>Phase 5 — Loop Outputs</t>
-        </is>
-      </c>
-      <c r="D167" t="inlineStr">
-        <is>
-          <t>Improvement</t>
-        </is>
-      </c>
-      <c r="E167" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="F167" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="G167" t="inlineStr">
-        <is>
-          <t>Baseball Analyst · Backend Developer</t>
-        </is>
-      </c>
-      <c r="H167" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="I167" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J167" t="inlineStr">
-        <is>
-          <t>prop TB is a lower bound (h+3·hr) until 2B/3B tracked.</t>
-        </is>
-      </c>
-      <c r="K167" t="inlineStr"/>
-      <c r="L167" t="inlineStr"/>
-      <c r="M167" t="inlineStr"/>
-      <c r="N167" t="inlineStr"/>
-    </row>
-    <row r="168">
-      <c r="A168" t="inlineStr">
-        <is>
-          <t>SIM-366</t>
-        </is>
-      </c>
-      <c r="B168" t="inlineStr">
-        <is>
-          <t>Per-player 100-iteration boxscore-average API shape (PropDistributionSet means)</t>
-        </is>
-      </c>
-      <c r="C168" t="inlineStr">
-        <is>
-          <t>Phase 5 — Backend API</t>
-        </is>
-      </c>
-      <c r="D168" t="inlineStr">
-        <is>
-          <t>Feature</t>
-        </is>
-      </c>
-      <c r="E168" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="F168" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="G168" t="inlineStr">
-        <is>
-          <t>Backend Developer · UX Designer</t>
-        </is>
-      </c>
-      <c r="H168" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="I168" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J168" t="inlineStr"/>
-      <c r="K168" t="inlineStr"/>
-      <c r="L168" t="inlineStr"/>
-      <c r="M168" t="inlineStr">
-        <is>
-          <t>SIM-350</t>
-        </is>
-      </c>
-      <c r="N168" t="inlineStr"/>
-    </row>
-    <row r="169">
-      <c r="A169" t="inlineStr">
-        <is>
-          <t>SIM-367</t>
-        </is>
-      </c>
-      <c r="B169" t="inlineStr">
-        <is>
-          <t>Run-line / spread EdgeReport from raw score-margin arrays</t>
-        </is>
-      </c>
-      <c r="C169" t="inlineStr">
-        <is>
-          <t>Phase 5 — Betting</t>
-        </is>
-      </c>
-      <c r="D169" t="inlineStr">
-        <is>
-          <t>Gap</t>
-        </is>
-      </c>
-      <c r="E169" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="F169" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="G169" t="inlineStr">
-        <is>
-          <t>Betting Analyst · ML Engineer</t>
-        </is>
-      </c>
-      <c r="H169" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="I169" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J169" t="inlineStr">
-        <is>
-          <t>Only ML/total/prop edge exist.</t>
-        </is>
-      </c>
-      <c r="K169" t="inlineStr"/>
-      <c r="L169" t="inlineStr"/>
-      <c r="M169" t="inlineStr"/>
-      <c r="N169" t="inlineStr"/>
-    </row>
-    <row r="170">
-      <c r="A170" t="inlineStr">
-        <is>
-          <t>SIM-368</t>
-        </is>
-      </c>
-      <c r="B170" t="inlineStr">
-        <is>
-          <t>CLV / line-movement time-series surface (opening→closing)</t>
-        </is>
-      </c>
-      <c r="C170" t="inlineStr">
-        <is>
-          <t>Phase 5 — Betting</t>
-        </is>
-      </c>
-      <c r="D170" t="inlineStr">
-        <is>
-          <t>Gap</t>
-        </is>
-      </c>
-      <c r="E170" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="F170" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="G170" t="inlineStr">
-        <is>
-          <t>Betting Analyst · Data Engineer</t>
-        </is>
-      </c>
-      <c r="H170" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="I170" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J170" t="inlineStr">
-        <is>
-          <t>CLV is a single entry-vs-close snapshot today.</t>
-        </is>
-      </c>
-      <c r="K170" t="inlineStr"/>
-      <c r="L170" t="inlineStr"/>
-      <c r="M170" t="inlineStr">
-        <is>
-          <t>SIM-370</t>
-        </is>
-      </c>
-      <c r="N170" t="inlineStr"/>
-    </row>
-    <row r="171">
-      <c r="A171" t="inlineStr">
-        <is>
-          <t>SIM-369</t>
-        </is>
-      </c>
-      <c r="B171" t="inlineStr">
-        <is>
-          <t>Bet-signal / +EV recommendation endpoint contract</t>
-        </is>
-      </c>
-      <c r="C171" t="inlineStr">
-        <is>
-          <t>Phase 5 — Betting</t>
-        </is>
-      </c>
-      <c r="D171" t="inlineStr">
-        <is>
-          <t>Feature</t>
-        </is>
-      </c>
-      <c r="E171" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="F171" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="G171" t="inlineStr">
-        <is>
-          <t>Betting Analyst</t>
-        </is>
-      </c>
-      <c r="H171" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="I171" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J171" t="inlineStr">
-        <is>
-          <t>Aggregate EdgeReports into a fireable signal.</t>
-        </is>
-      </c>
-      <c r="K171" t="inlineStr"/>
-      <c r="L171" t="inlineStr"/>
-      <c r="M171" t="inlineStr">
-        <is>
-          <t>SIM-367</t>
-        </is>
-      </c>
-      <c r="N171" t="inlineStr"/>
-    </row>
-    <row r="172">
-      <c r="A172" t="inlineStr">
-        <is>
-          <t>SIM-370</t>
-        </is>
-      </c>
-      <c r="B172" t="inlineStr">
-        <is>
-          <t>Real odds/prop provider swap behind MockOddsAPI</t>
-        </is>
-      </c>
-      <c r="C172" t="inlineStr">
-        <is>
-          <t>Phase 5 — Betting</t>
-        </is>
-      </c>
-      <c r="D172" t="inlineStr">
-        <is>
-          <t>Feature</t>
-        </is>
-      </c>
-      <c r="E172" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="F172" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="G172" t="inlineStr">
-        <is>
-          <t>Data Engineer · Betting Analyst</t>
-        </is>
-      </c>
-      <c r="H172" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="I172" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J172" t="inlineStr">
-        <is>
-          <t>Multi-book, sharp flag; cadence wired by SIM-340.</t>
-        </is>
-      </c>
-      <c r="K172" t="inlineStr"/>
-      <c r="L172" t="inlineStr"/>
-      <c r="M172" t="inlineStr"/>
-      <c r="N172" t="inlineStr"/>
-    </row>
-    <row r="173">
-      <c r="A173" t="inlineStr">
-        <is>
-          <t>SIM-371</t>
-        </is>
-      </c>
-      <c r="B173" t="inlineStr">
-        <is>
-          <t>API integration + WebSocket + historical-replay E2E suite</t>
-        </is>
-      </c>
-      <c r="C173" t="inlineStr">
-        <is>
-          <t>Phase 5 — Testing</t>
-        </is>
-      </c>
-      <c r="D173" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
-      <c r="E173" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="F173" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="G173" t="inlineStr">
-        <is>
-          <t>QA/DevOps · Baseball Analyst</t>
-        </is>
-      </c>
-      <c r="H173" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="I173" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J173" t="inlineStr">
-        <is>
-          <t>api/websocket/ is an empty placeholder.</t>
-        </is>
-      </c>
-      <c r="K173" t="inlineStr"/>
-      <c r="L173" t="inlineStr"/>
-      <c r="M173" t="inlineStr">
-        <is>
-          <t>SIM-355</t>
-        </is>
-      </c>
-      <c r="N173" t="inlineStr"/>
-    </row>
-    <row r="174">
-      <c r="A174" t="inlineStr">
-        <is>
-          <t>SIM-372</t>
-        </is>
-      </c>
-      <c r="B174" t="inlineStr">
-        <is>
-          <t>End-to-end /simulate latency perf gate (2s/30s SLA)</t>
-        </is>
-      </c>
-      <c r="C174" t="inlineStr">
-        <is>
-          <t>Phase 5 — Testing</t>
-        </is>
-      </c>
-      <c r="D174" t="inlineStr">
-        <is>
-          <t>Perf</t>
-        </is>
-      </c>
-      <c r="E174" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="F174" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="G174" t="inlineStr">
-        <is>
-          <t>Performance Engineer</t>
-        </is>
-      </c>
-      <c r="H174" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="I174" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J174" t="inlineStr">
-        <is>
-          <t>Current bench skips the request path.</t>
-        </is>
-      </c>
-      <c r="K174" t="inlineStr"/>
-      <c r="L174" t="inlineStr"/>
-      <c r="M174" t="inlineStr">
-        <is>
-          <t>SIM-352</t>
-        </is>
-      </c>
-      <c r="N174" t="inlineStr"/>
-    </row>
-    <row r="175">
-      <c r="A175" t="inlineStr">
-        <is>
-          <t>SIM-373</t>
-        </is>
-      </c>
-      <c r="B175" t="inlineStr">
-        <is>
-          <t>nginx reverse proxy w/ WebSocket upgrade + dev/staging/prod env configs</t>
-        </is>
-      </c>
-      <c r="C175" t="inlineStr">
-        <is>
-          <t>Phase 5 — Infra</t>
-        </is>
-      </c>
-      <c r="D175" t="inlineStr">
-        <is>
-          <t>Infra</t>
-        </is>
-      </c>
-      <c r="E175" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="F175" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="G175" t="inlineStr">
-        <is>
-          <t>QA/DevOps</t>
-        </is>
-      </c>
-      <c r="H175" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="I175" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J175" t="inlineStr"/>
-      <c r="K175" t="inlineStr"/>
-      <c r="L175" t="inlineStr"/>
-      <c r="M175" t="inlineStr">
-        <is>
-          <t>SIM-354</t>
-        </is>
-      </c>
-      <c r="N175" t="inlineStr"/>
-    </row>
-    <row r="176">
-      <c r="A176" t="inlineStr">
-        <is>
-          <t>SIM-374</t>
-        </is>
-      </c>
-      <c r="B176" t="inlineStr">
-        <is>
-          <t>Prometheus + Grafana monitoring (sim latency, API p95, pipeline freshness)</t>
-        </is>
-      </c>
-      <c r="C176" t="inlineStr">
-        <is>
-          <t>Phase 5 — Infra</t>
-        </is>
-      </c>
-      <c r="D176" t="inlineStr">
-        <is>
-          <t>Infra</t>
-        </is>
-      </c>
-      <c r="E176" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="F176" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="G176" t="inlineStr">
-        <is>
-          <t>QA/DevOps</t>
-        </is>
-      </c>
-      <c r="H176" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="I176" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J176" t="inlineStr"/>
-      <c r="K176" t="inlineStr"/>
-      <c r="L176" t="inlineStr"/>
-      <c r="M176" t="inlineStr">
-        <is>
-          <t>SIM-373</t>
-        </is>
-      </c>
-      <c r="N176" t="inlineStr"/>
-    </row>
-    <row r="177">
-      <c r="A177" t="inlineStr">
-        <is>
-          <t>SIM-375</t>
-        </is>
-      </c>
-      <c r="B177" t="inlineStr">
-        <is>
-          <t>Fix docker-compose.yml to mount ./simulation + remove the dead simulator/ package</t>
-        </is>
-      </c>
-      <c r="C177" t="inlineStr">
-        <is>
-          <t>Phase 5 — Infra</t>
-        </is>
-      </c>
-      <c r="D177" t="inlineStr">
-        <is>
-          <t>Bug</t>
-        </is>
-      </c>
-      <c r="E177" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="F177" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="G177" t="inlineStr">
-        <is>
-          <t>Data Engineer · QA/DevOps</t>
-        </is>
-      </c>
-      <c r="H177" t="inlineStr">
+      <c r="H179" s="46" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
       </c>
-      <c r="I177" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J177" t="inlineStr">
-        <is>
-          <t>Compose mounted the empty ./simulator stub.</t>
-        </is>
-      </c>
-      <c r="K177" t="inlineStr">
-        <is>
-          <t>compose mounts ./simulation; Dockerfile copies simulation/+betting/; simulator/ deleted.</t>
-        </is>
-      </c>
-      <c r="L177" t="inlineStr"/>
-      <c r="M177" t="inlineStr">
-        <is>
-          <t>Closed 2026-05-24 (Sprint 1).</t>
-        </is>
-      </c>
-    </row>
-    <row r="178">
-      <c r="A178" t="inlineStr">
-        <is>
-          <t>SIM-376</t>
-        </is>
-      </c>
-      <c r="B178" t="inlineStr">
-        <is>
-          <t>Add api/ to the coverage gate (pyproject source + ci --cov=api)</t>
-        </is>
-      </c>
-      <c r="C178" t="inlineStr">
-        <is>
-          <t>Phase 5 — Infra</t>
-        </is>
-      </c>
-      <c r="D178" t="inlineStr">
-        <is>
-          <t>Bug</t>
-        </is>
-      </c>
-      <c r="E178" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="F178" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="G178" t="inlineStr">
-        <is>
-          <t>QA/DevOps</t>
-        </is>
-      </c>
-      <c r="H178" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="I178" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J178" t="inlineStr">
-        <is>
-          <t>Only the Makefile measured api/ coverage.</t>
-        </is>
-      </c>
-      <c r="K178" t="inlineStr">
-        <is>
-          <t>pyproject source += api; ci --cov=api.</t>
-        </is>
-      </c>
-      <c r="L178" t="inlineStr"/>
-      <c r="M178" t="inlineStr">
-        <is>
-          <t>Closed 2026-05-24 (Sprint 1).</t>
-        </is>
-      </c>
-    </row>
-    <row r="179">
-      <c r="A179" t="inlineStr">
-        <is>
-          <t>SIM-377</t>
-        </is>
-      </c>
-      <c r="B179" t="inlineStr">
-        <is>
-          <t>Fix/remove GameSpec._hit_rate (factory reads it but simulate_game has no **kwargs → TypeError)</t>
-        </is>
-      </c>
-      <c r="C179" t="inlineStr">
-        <is>
-          <t>Phase 5 — Infra</t>
-        </is>
-      </c>
-      <c r="D179" t="inlineStr">
-        <is>
-          <t>Bug</t>
-        </is>
-      </c>
-      <c r="E179" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="F179" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="G179" t="inlineStr">
-        <is>
-          <t>Backend Developer</t>
-        </is>
-      </c>
-      <c r="H179" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="I179" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J179" t="inlineStr">
+      <c r="I179" s="46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J179" s="46" t="inlineStr">
         <is>
           <t>_hit_rate splatted into simulate_game raised TypeError.</t>
         </is>
       </c>
-      <c r="K179" t="inlineStr">
+      <c r="K179" s="46" t="inlineStr">
         <is>
           <t>_run_one filters _-prefixed factory-only keys.</t>
         </is>
       </c>
-      <c r="L179" t="inlineStr"/>
-      <c r="M179" t="inlineStr">
+      <c r="L179" s="46" t="inlineStr"/>
+      <c r="M179" s="46" t="inlineStr">
         <is>
           <t>Closed 2026-05-24 (Sprint 1). 7 tests.</t>
         </is>

</xml_diff>

<commit_message>
Phase 5 Sprint 3 - P1 lifecycle (SIM-360 persistent pool + SIM-361 calibration/11-engine startup); P1 tier complete; suite 1702 green
</commit_message>
<xml_diff>
--- a/backlog.xlsx
+++ b/backlog.xlsx
@@ -15712,7 +15712,7 @@
       </c>
       <c r="H162" s="46" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="I162" s="46" t="inlineStr">
@@ -15729,7 +15729,7 @@
       <c r="L162" s="46" t="inlineStr"/>
       <c r="M162" s="46" t="inlineStr">
         <is>
-          <t>SIM-352</t>
+          <t>SIM-352 | Closed 2026-05-24 (Phase 5 Sprint 3; P1 tier complete).</t>
         </is>
       </c>
       <c r="N162" s="46" t="inlineStr"/>
@@ -15772,7 +15772,7 @@
       </c>
       <c r="H163" s="46" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="I163" s="46" t="inlineStr">
@@ -15787,7 +15787,11 @@
       </c>
       <c r="K163" s="46" t="inlineStr"/>
       <c r="L163" s="46" t="inlineStr"/>
-      <c r="M163" s="46" t="inlineStr"/>
+      <c r="M163" s="46" t="inlineStr">
+        <is>
+          <t>Closed 2026-05-24 (Phase 5 Sprint 3; P1 tier complete).</t>
+        </is>
+      </c>
       <c r="N163" s="46" t="inlineStr"/>
     </row>
     <row r="164">

</xml_diff>

<commit_message>
Phase 5 Sprint 5 - betting surface (SIM-367 spread edge, 368 CLV/line-movement, 369 bet-signals, 370 odds provider) + /api/betting router; suite 1861 green
</commit_message>
<xml_diff>
--- a/backlog.xlsx
+++ b/backlog.xlsx
@@ -15832,7 +15832,7 @@
       </c>
       <c r="H164" s="46" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="I164" s="46" t="inlineStr">
@@ -15847,7 +15847,11 @@
       </c>
       <c r="K164" s="46" t="inlineStr"/>
       <c r="L164" s="46" t="inlineStr"/>
-      <c r="M164" s="46" t="inlineStr"/>
+      <c r="M164" s="46" t="inlineStr">
+        <is>
+          <t>Closed 2026-05-24 (Phase 5 Sprint 4).</t>
+        </is>
+      </c>
       <c r="N164" s="46" t="inlineStr"/>
     </row>
     <row r="165">
@@ -15888,7 +15892,7 @@
       </c>
       <c r="H165" s="46" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="I165" s="46" t="inlineStr">
@@ -15905,7 +15909,7 @@
       <c r="L165" s="46" t="inlineStr"/>
       <c r="M165" s="46" t="inlineStr">
         <is>
-          <t>SIM-353</t>
+          <t>SIM-353 | Closed 2026-05-24 (Phase 5 Sprint 4).</t>
         </is>
       </c>
       <c r="N165" s="46" t="inlineStr"/>
@@ -15948,7 +15952,7 @@
       </c>
       <c r="H166" s="46" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="I166" s="46" t="inlineStr">
@@ -15965,7 +15969,7 @@
       <c r="L166" s="46" t="inlineStr"/>
       <c r="M166" s="46" t="inlineStr">
         <is>
-          <t>SIM-362</t>
+          <t>SIM-362 | Closed 2026-05-24 (Phase 5 Sprint 4).</t>
         </is>
       </c>
       <c r="N166" s="46" t="inlineStr"/>
@@ -16008,7 +16012,7 @@
       </c>
       <c r="H167" s="46" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="I167" s="46" t="inlineStr">
@@ -16023,7 +16027,11 @@
       </c>
       <c r="K167" s="46" t="inlineStr"/>
       <c r="L167" s="46" t="inlineStr"/>
-      <c r="M167" s="46" t="inlineStr"/>
+      <c r="M167" s="46" t="inlineStr">
+        <is>
+          <t>Closed 2026-05-24 (Phase 5 Sprint 4).</t>
+        </is>
+      </c>
       <c r="N167" s="46" t="inlineStr"/>
     </row>
     <row r="168">
@@ -16064,7 +16072,7 @@
       </c>
       <c r="H168" s="46" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="I168" s="46" t="inlineStr">
@@ -16077,7 +16085,7 @@
       <c r="L168" s="46" t="inlineStr"/>
       <c r="M168" s="46" t="inlineStr">
         <is>
-          <t>SIM-350</t>
+          <t>SIM-350 | Closed 2026-05-24 (Phase 5 Sprint 4).</t>
         </is>
       </c>
       <c r="N168" s="46" t="inlineStr"/>
@@ -16120,7 +16128,7 @@
       </c>
       <c r="H169" s="46" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="I169" s="46" t="inlineStr">
@@ -16135,7 +16143,11 @@
       </c>
       <c r="K169" s="46" t="inlineStr"/>
       <c r="L169" s="46" t="inlineStr"/>
-      <c r="M169" s="46" t="inlineStr"/>
+      <c r="M169" s="46" t="inlineStr">
+        <is>
+          <t>Closed 2026-05-24 (Phase 5 Sprint 5; betting surface + /api/betting).</t>
+        </is>
+      </c>
       <c r="N169" s="46" t="inlineStr"/>
     </row>
     <row r="170">
@@ -16176,7 +16188,7 @@
       </c>
       <c r="H170" s="46" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="I170" s="46" t="inlineStr">
@@ -16193,7 +16205,7 @@
       <c r="L170" s="46" t="inlineStr"/>
       <c r="M170" s="46" t="inlineStr">
         <is>
-          <t>SIM-370</t>
+          <t>SIM-370 | Closed 2026-05-24 (Phase 5 Sprint 5; betting surface + /api/betting).</t>
         </is>
       </c>
       <c r="N170" s="46" t="inlineStr"/>
@@ -16236,7 +16248,7 @@
       </c>
       <c r="H171" s="46" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="I171" s="46" t="inlineStr">
@@ -16253,7 +16265,7 @@
       <c r="L171" s="46" t="inlineStr"/>
       <c r="M171" s="46" t="inlineStr">
         <is>
-          <t>SIM-367</t>
+          <t>SIM-367 | Closed 2026-05-24 (Phase 5 Sprint 5; betting surface + /api/betting).</t>
         </is>
       </c>
       <c r="N171" s="46" t="inlineStr"/>
@@ -16296,7 +16308,7 @@
       </c>
       <c r="H172" s="46" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="I172" s="46" t="inlineStr">
@@ -16311,7 +16323,11 @@
       </c>
       <c r="K172" s="46" t="inlineStr"/>
       <c r="L172" s="46" t="inlineStr"/>
-      <c r="M172" s="46" t="inlineStr"/>
+      <c r="M172" s="46" t="inlineStr">
+        <is>
+          <t>Closed 2026-05-24 (Phase 5 Sprint 5; betting surface + /api/betting).</t>
+        </is>
+      </c>
       <c r="N172" s="46" t="inlineStr"/>
     </row>
     <row r="173">

</xml_diff>

<commit_message>
Phase 5 Sprint 6 - testing/infra (SIM-371 E2E/WS suite, 372 /simulate SLA gate, 373 nginx, 374 monitoring); PHASE 5 COMPLETE; suite 1870 green
</commit_message>
<xml_diff>
--- a/backlog.xlsx
+++ b/backlog.xlsx
@@ -16368,7 +16368,7 @@
       </c>
       <c r="H173" s="46" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="I173" s="46" t="inlineStr">
@@ -16385,7 +16385,7 @@
       <c r="L173" s="46" t="inlineStr"/>
       <c r="M173" s="46" t="inlineStr">
         <is>
-          <t>SIM-355</t>
+          <t>SIM-355 | Closed 2026-05-24 (Phase 5 Sprint 6; PHASE 5 COMPLETE).</t>
         </is>
       </c>
       <c r="N173" s="46" t="inlineStr"/>
@@ -16428,7 +16428,7 @@
       </c>
       <c r="H174" s="46" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="I174" s="46" t="inlineStr">
@@ -16445,7 +16445,7 @@
       <c r="L174" s="46" t="inlineStr"/>
       <c r="M174" s="46" t="inlineStr">
         <is>
-          <t>SIM-352</t>
+          <t>SIM-352 | Closed 2026-05-24 (Phase 5 Sprint 6; PHASE 5 COMPLETE).</t>
         </is>
       </c>
       <c r="N174" s="46" t="inlineStr"/>
@@ -16488,7 +16488,7 @@
       </c>
       <c r="H175" s="46" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="I175" s="46" t="inlineStr">
@@ -16501,7 +16501,7 @@
       <c r="L175" s="46" t="inlineStr"/>
       <c r="M175" s="46" t="inlineStr">
         <is>
-          <t>SIM-354</t>
+          <t>SIM-354 | Closed 2026-05-24 (Phase 5 Sprint 6; PHASE 5 COMPLETE).</t>
         </is>
       </c>
       <c r="N175" s="46" t="inlineStr"/>
@@ -16544,7 +16544,7 @@
       </c>
       <c r="H176" s="46" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="I176" s="46" t="inlineStr">
@@ -16557,7 +16557,7 @@
       <c r="L176" s="46" t="inlineStr"/>
       <c r="M176" s="46" t="inlineStr">
         <is>
-          <t>SIM-373</t>
+          <t>SIM-373 | Closed 2026-05-24 (Phase 5 Sprint 6; PHASE 5 COMPLETE).</t>
         </is>
       </c>
       <c r="N176" s="46" t="inlineStr"/>

</xml_diff>

<commit_message>
feat(sim-392): LinescoreGraphic + BaseballFieldGraphic SVG
- LinescoreGraphic: scoreboard R/H/E grid, "x" for unplayed halves, extra-inning widening (mirrors LinescoreModel SIM-362)
- BaseballFieldGraphic: SVG diamond, 9 fielder positions, occupied-base markers, runner + batter labels, label-collision rules
- graphics barrel export
Prop-driven; tsc + eslint pass. Wired into the Game page in SIM-393.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog.xlsx
+++ b/backlog.xlsx
@@ -2677,12 +2677,12 @@
       </c>
       <c r="H16" s="46" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="I16" s="46" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="J16" s="46" t="inlineStr">
@@ -20483,12 +20483,12 @@
       </c>
       <c r="H194" s="46" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="I194" s="46" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="J194" s="46" t="inlineStr">

</xml_diff>

<commit_message>
feat(sim-393): Game page (linescore + field + play-by-play + live WS)
- GamePage at /game/:gamePk: header (matchup + status + score), live banner
  (WS status + re-sim indicator), linescore + field graphics, play-by-play,
  slots for projections (SIM-394) + betting (SIM-395)
- useGameSocket hook: /ws/games/{pk} subscription, SIM-385 events
  (game_state_update / resim_pending / ping->pong), normalize runner fields,
  3s reconnect backoff
- PlayByPlayList: PA-grouped scroll + pitch drill-down
- games.ts: fetchLinescore / fetchPlays / fetchLiveState + types
- BaseballFieldGraphic: widen base props to string|boolean|null
404-tolerant fetches (no sim/not live = no data). tsc + eslint + build pass.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog.xlsx
+++ b/backlog.xlsx
@@ -2744,12 +2744,12 @@
       </c>
       <c r="H17" s="46" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="I17" s="46" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="J17" s="46" t="inlineStr">
@@ -20550,12 +20550,12 @@
       </c>
       <c r="H195" s="46" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="I195" s="46" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="J195" s="46" t="inlineStr">

</xml_diff>

<commit_message>
feat(sim-394): per-player boxscore means + prop distribution chart
- BoxscorePanel: "Load projections" gate -> /boxscore means as prop chips;
  select a chip -> fetch PMF (SIM-390) -> distribution chart + line input
  (P(over)/P(under)/P(push))
- PropDistributionChart: SVG PMF bars + dashed prop-line marker + mean marker + over-bar tint
- games.ts: fetchBoxscore + fetchPropEdge (line/odds/bet_side params) + types
- GamePage: mount BoxscorePanel in the Projections slot
tsc + eslint + build pass.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog.xlsx
+++ b/backlog.xlsx
@@ -2811,12 +2811,12 @@
       </c>
       <c r="H18" s="46" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="I18" s="46" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="J18" s="46" t="inlineStr">
@@ -20617,12 +20617,12 @@
       </c>
       <c r="H196" s="46" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="I196" s="46" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="J196" s="46" t="inlineStr">

</xml_diff>

<commit_message>
feat(sim-395): betting card surface (edges + signals + odds_source)
- api/betting.ts: fetchEdges / fetchSignals / fetchLineMovement + types
- BettingCard: per-market (ML/total/run-line) edges, favored-side highlight,
  +EV signal badge (stake% + offered price), mock-vs-live odds_source flag;
  gated behind "Load betting"
- GamePage: mount BettingCard in the Betting slot
tsc + eslint + build pass.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog.xlsx
+++ b/backlog.xlsx
@@ -2878,12 +2878,12 @@
       </c>
       <c r="H19" s="46" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="I19" s="46" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="J19" s="46" t="inlineStr">
@@ -20684,12 +20684,12 @@
       </c>
       <c r="H197" s="46" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="I197" s="46" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="J197" s="46" t="inlineStr">

</xml_diff>

<commit_message>
feat(sim-396): CLV / line-movement time-series chart
- LineMovementChart: SVG implied-prob series (open->close), close marker,
  sharp/steam/beat-close badges, CLV% footer
- LineMovementPanel: market tabs (ML/total/run-line), fetch /line-movement on
  mount, chart per (side,book) series, empty-history message
- GamePage: mount LineMovementPanel
tsc + eslint + build pass.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog.xlsx
+++ b/backlog.xlsx
@@ -2945,12 +2945,12 @@
       </c>
       <c r="H20" s="46" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="I20" s="46" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="J20" s="46" t="inlineStr">
@@ -20751,12 +20751,12 @@
       </c>
       <c r="H198" s="46" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="I198" s="46" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="J198" s="46" t="inlineStr">

</xml_diff>

<commit_message>
feat(sim-397): managerial override UI v1 (single-sub)
- OverridePanelV1: single-sub form -> POST /simulate/with_override -> delta
- OverrideDeltaView: shared baseline/override/delta table (reused by SIM-398)
- games.ts: postWithOverride + postJson + override types
- GamePage: mount OverridePanelV1
tsc + eslint + build pass.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog.xlsx
+++ b/backlog.xlsx
@@ -3012,12 +3012,12 @@
       </c>
       <c r="H21" s="46" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="I21" s="46" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="J21" s="46" t="inlineStr">
@@ -20818,12 +20818,12 @@
       </c>
       <c r="H199" s="46" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="I199" s="46" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="J199" s="46" t="inlineStr">

</xml_diff>

<commit_message>
feat(sim-398): managerial override UI v2 (staged queue + undo + multi-change)
- OverridePanelV2: stage N substitutions, undo per row, clear all, run together
  via substitutions[] (SIM-388); amber "override active" badge; side-by-side
  baseline/override result
- GamePage: override panel now mounts V2 (supersedes V1)
tsc + eslint + build pass.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog.xlsx
+++ b/backlog.xlsx
@@ -3079,12 +3079,12 @@
       </c>
       <c r="H22" s="46" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="I22" s="46" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="J22" s="46" t="inlineStr">
@@ -20885,12 +20885,12 @@
       </c>
       <c r="H200" s="46" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="I200" s="46" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="J200" s="46" t="inlineStr">

</xml_diff>

<commit_message>
feat(sim-399): a11y + responsive pass
- global.css: :focus-visible ring, prefers-reduced-motion, .skip-link,
  responsive header (<=640px); removed dead .placeholder-card + double
  width/padding on .app-main
- App.tsx: skip-to-content link
Cross-browser verification deferred to SIM-400 live run. tsc + eslint + build pass.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog.xlsx
+++ b/backlog.xlsx
@@ -3146,12 +3146,12 @@
       </c>
       <c r="H23" s="46" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="I23" s="46" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="J23" s="46" t="inlineStr">
@@ -20952,12 +20952,12 @@
       </c>
       <c r="H201" s="46" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="I201" s="46" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="J201" s="46" t="inlineStr">

</xml_diff>

<commit_message>
test(sim-400): Playwright cross-browser E2E harness + smoke specs
- playwright.config.ts: chromium/firefox/webkit projects + webServer (build+preview :4173)
- e2e/smoke.spec.ts: 4 backend-mocked smoke tests (login gate, slate render,
  card->game nav, date nav) — no live API/DB needed
- package.json: @playwright/test + e2e / e2e:install scripts (lock regenerated)
- ci.yml: frontend-e2e job (install browsers, run all 3 engines, upload report)
- .gitignore: playwright artifacts

Verified: chromium project ran locally, 4/4 passed (first real browser
verification of the frontend). firefox/webkit run in CI.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog.xlsx
+++ b/backlog.xlsx
@@ -3213,12 +3213,12 @@
       </c>
       <c r="H24" s="46" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="I24" s="46" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="J24" s="46" t="inlineStr">
@@ -21019,12 +21019,12 @@
       </c>
       <c r="H202" s="46" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="I202" s="46" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="J202" s="46" t="inlineStr">

</xml_diff>

<commit_message>
feat(sim-401): frontend deploy (Docker image + nginx + CD to ghcr)
- frontend/Dockerfile: multi-stage (node build -> nginx serving the SPA from
  /var/www/baseball-sim + shared SIM-381 nginx.conf reverse proxy)
- frontend/Dockerfile.dockerignore: BuildKit adjacent ignore overriding the
  root .dockerignore (keeps frontend/ + deploy/nginx/ in context)
- frontend-release.yml: CD pushing ghcr.io/<repo>-frontend (:sha/:latest/semver)
- docker-compose.yml: nginx service now builds frontend/Dockerfile; healthcheck -> /index.html

Verified: docker build succeeds; baked image has /var/www/baseball-sim/index.html
+ assets + matching nginx root. Sprint 2 (P1 frontend build) COMPLETE: SIM-391->401.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog.xlsx
+++ b/backlog.xlsx
@@ -3280,12 +3280,12 @@
       </c>
       <c r="H25" s="46" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="I25" s="46" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="J25" s="46" t="inlineStr">
@@ -21086,12 +21086,12 @@
       </c>
       <c r="H203" s="46" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="I203" s="46" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="J203" s="46" t="inlineStr">

</xml_diff>

<commit_message>
docs: close SIM-415/416/417/418/419/420 (P1/P2 hardening batch)
CHANGES.md hardening-batch section + per-ticket detail; BACKLOG.md banner +
rows marked Closed; backlog.xlsx (31 closed / 12 open). Verified: 113 tests
green across new + touched suites.

Remaining Phase 6: P1 data/ML/perf SIM-402->409 (live-env), P2 sim-realism
SIM-411->414, and SIM-405 (BettingPros odds provider) next.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog.xlsx
+++ b/backlog.xlsx
@@ -4188,7 +4188,7 @@
       </c>
       <c r="H39" s="46" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="I39" s="46" t="inlineStr">
@@ -4250,7 +4250,7 @@
       </c>
       <c r="H40" s="46" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="I40" s="46" t="inlineStr">
@@ -4312,7 +4312,7 @@
       </c>
       <c r="H41" s="46" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="I41" s="46" t="inlineStr">
@@ -4374,7 +4374,7 @@
       </c>
       <c r="H42" s="46" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="I42" s="46" t="inlineStr">
@@ -4436,7 +4436,7 @@
       </c>
       <c r="H43" s="46" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="I43" s="46" t="inlineStr">
@@ -4498,12 +4498,12 @@
       </c>
       <c r="H44" s="46" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="I44" s="46" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="J44" s="46" t="inlineStr">
@@ -21994,7 +21994,7 @@
       </c>
       <c r="H217" s="46" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="I217" s="46" t="inlineStr">
@@ -22056,7 +22056,7 @@
       </c>
       <c r="H218" s="46" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="I218" s="46" t="inlineStr">
@@ -22118,7 +22118,7 @@
       </c>
       <c r="H219" s="46" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="I219" s="46" t="inlineStr">
@@ -22180,7 +22180,7 @@
       </c>
       <c r="H220" s="46" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="I220" s="46" t="inlineStr">
@@ -22242,7 +22242,7 @@
       </c>
       <c r="H221" s="46" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="I221" s="46" t="inlineStr">
@@ -22304,12 +22304,12 @@
       </c>
       <c r="H222" s="46" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="I222" s="46" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="J222" s="46" t="inlineStr">

</xml_diff>

<commit_message>
docs(backlog): add SIM-421 — full book-offered market projection (P3, future)
Non-essential future enhancement: extend the simulator's prop/market projection
beyond the core 8 props + 3 game markets to the full set the book offers and the
pitch-by-pitch sim can derive — individual hit types (1B/2B/3B), SB,
hits/walks-allowed, H+R+RBI combos, per-team totals, first-five-innings
ML/RL/total, and NRFI/YRFI. Mostly computable from existing per-iteration output;
wire to the prop-edge surface + BettingPros market map, then calibrate.

- new "Tier P3 — future enhancements (post-stabilization)" in BACKLOG.md
- depends-on SIM-402/406/407 (core live-env verified + calibrated first)
- backlog.xlsx Full Backlog + Phase 6 Build rows
- next free ticket ID bumped to SIM-422 (BACKLOG.md + CLAUDE.md)

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog.xlsx
+++ b/backlog.xlsx
@@ -1652,7 +1652,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:M44"/>
+  <dimension ref="A1:M45"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.71484375" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="11" customWidth="1" style="46" min="1" max="1"/>
@@ -4524,6 +4524,73 @@
       <c r="M44" s="46" t="inlineStr">
         <is>
           <t>Tier P2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>SIM-421</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Extend prop/market projection to the full book-offered market set</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Simulation</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>ML Engineer + Baseball Analyst + Betting Analyst</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>The sim projects 8 player props (K/BB/ER/OUTS, H/HR/RBI/TB) + 3 game markets (moneyline/total/run-line). The book (BettingPros, SIM-405) offers many more that are derivable from the existing pitch-by-pitch simulation: individual hit types (singles 1B / doubles 2B / triples 3B), stolen bases, hits-allowed / walks-allowed, hits+runs+RBIs combos; and game derivatives - per-team run totals, first-five-innings (F5) moneyline/run-line/total, and no-runs-first-inning (NRFI/YRFI). Most are computable from existing per-iteration output (the boxscore already tracks 1B/2B/3B; inning-by-inning scores give F5 + first-inning runs), so the work is mainly computing the PMFs/distributions from existing sim state and wiring them to the prop-edge surface + the BettingPros market map, then calibrating.</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>New prop/market PMFs computed from the 100-iteration run and exposed via the prop-edge endpoint (SIM-390 pattern); mapped to the corresponding BettingPros market ids (SIM-405); calibrated (no uncalibrated numbers reach users); unit tests for each new market family.</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>SIM-402, SIM-406, SIM-407</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>NON-ESSENTIAL future enhancement. Deferred until the core 8-prop / 3-market surface is live-env verified + calibrated (SIM-402/406/407) and the project is in a stable spot. Requested 2026-05-26.</t>
         </is>
       </c>
     </row>
@@ -7435,7 +7502,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:N222"/>
+  <dimension ref="A1:N223"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.71484375" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="11" customWidth="1" style="46" min="1" max="1"/>
@@ -22330,6 +22397,73 @@
       <c r="M222" s="46" t="inlineStr">
         <is>
           <t>Tier P2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>SIM-421</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>Extend prop/market projection to the full book-offered market set</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>Simulation</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="F223" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G223" t="inlineStr">
+        <is>
+          <t>ML Engineer + Baseball Analyst + Betting Analyst</t>
+        </is>
+      </c>
+      <c r="H223" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I223" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J223" t="inlineStr">
+        <is>
+          <t>The sim projects 8 player props (K/BB/ER/OUTS, H/HR/RBI/TB) + 3 game markets (moneyline/total/run-line). The book (BettingPros, SIM-405) offers many more that are derivable from the existing pitch-by-pitch simulation: individual hit types (singles 1B / doubles 2B / triples 3B), stolen bases, hits-allowed / walks-allowed, hits+runs+RBIs combos; and game derivatives - per-team run totals, first-five-innings (F5) moneyline/run-line/total, and no-runs-first-inning (NRFI/YRFI). Most are computable from existing per-iteration output (the boxscore already tracks 1B/2B/3B; inning-by-inning scores give F5 + first-inning runs), so the work is mainly computing the PMFs/distributions from existing sim state and wiring them to the prop-edge surface + the BettingPros market map, then calibrating.</t>
+        </is>
+      </c>
+      <c r="K223" t="inlineStr">
+        <is>
+          <t>New prop/market PMFs computed from the 100-iteration run and exposed via the prop-edge endpoint (SIM-390 pattern); mapped to the corresponding BettingPros market ids (SIM-405); calibrated (no uncalibrated numbers reach users); unit tests for each new market family.</t>
+        </is>
+      </c>
+      <c r="L223" t="inlineStr">
+        <is>
+          <t>SIM-402, SIM-406, SIM-407</t>
+        </is>
+      </c>
+      <c r="M223" t="inlineStr">
+        <is>
+          <t>NON-ESSENTIAL future enhancement. Deferred until the core 8-prop / 3-market surface is live-env verified + calibrated (SIM-402/406/407) and the project is in a stable spot. Requested 2026-05-26.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(sim-436): file low-priority ticket to revisit /simulate perf for the 30s SLA
SIM-430's forkserver fix cleared the OOM (n=100 215s→~38s) but the 30s batch SLA
is not met and throughput plateaus past ~6 workers (a serial parent-side
result-collection/aggregation + per-request machine-rebuild bottleneck, not a
worker-count one). SIM-436 (P3/low) tracks revisiting per-game cost + fan-out
efficiency to land <30s. Low priority — simulations already run at scale (no OOM).
Next free ID → SIM-437.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog.xlsx
+++ b/backlog.xlsx
@@ -7502,7 +7502,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:N238"/>
+  <dimension ref="A1:N239"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.71484375" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="11" customWidth="1" style="46" min="1" max="1"/>
@@ -23469,6 +23469,73 @@
       <c r="M238" s="46" t="inlineStr">
         <is>
           <t>Filed 2026-06-01.</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="46" t="inlineStr">
+        <is>
+          <t>SIM-436</t>
+        </is>
+      </c>
+      <c r="B239" s="46" t="inlineStr">
+        <is>
+          <t>Revisit /simulate per-game cost + fan-out efficiency to meet the 30s SLA</t>
+        </is>
+      </c>
+      <c r="C239" s="46" t="inlineStr">
+        <is>
+          <t>Phase 7 - Perf</t>
+        </is>
+      </c>
+      <c r="D239" s="46" t="inlineStr">
+        <is>
+          <t>Perf</t>
+        </is>
+      </c>
+      <c r="E239" s="46" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="F239" s="46" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="G239" s="46" t="inlineStr">
+        <is>
+          <t>Performance Engineer + Backend Developer</t>
+        </is>
+      </c>
+      <c r="H239" s="46" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I239" s="46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J239" s="46" t="inlineStr">
+        <is>
+          <t>SIM-430 forkserver fix cleared the OOM (n=100 215s-&gt;~38s) but the 30s SLA is not met and throughput plateaus past ~6 workers (serial bottleneck).</t>
+        </is>
+      </c>
+      <c r="K239" s="46" t="inlineStr">
+        <is>
+          <t>Profile parent-side result un-pickle + GameSimSummary aggregation + per-request StateMachine rebuild; land n=100 &lt; 30s. LOW priority - sims already run at scale.</t>
+        </is>
+      </c>
+      <c r="L239" s="46" t="inlineStr">
+        <is>
+          <t>SIM-430</t>
+        </is>
+      </c>
+      <c r="M239" s="46" t="inlineStr">
+        <is>
+          <t>Filed 2026-06-02. Polish to hit the stated SLA.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(sim-433/434/435): mark code-complete in CLAUDE + backlog.xlsx
CLAUDE §2a + the Full Backlog rows note the bullpen/manager/odds foundations are
code-complete (commit 812f0e8) with data-runs pending; record the SIM-436 perf
ticket + the build-cache/disk caution.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog.xlsx
+++ b/backlog.xlsx
@@ -23309,7 +23309,7 @@
       </c>
       <c r="H236" s="46" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Code-complete</t>
         </is>
       </c>
       <c r="I236" s="46" t="inlineStr">
@@ -23334,7 +23334,7 @@
       </c>
       <c r="M236" s="46" t="inlineStr">
         <is>
-          <t>Prerequisite for SIM-427 USAGE columns. Filed 2026-06-01.</t>
+          <t>Code-complete 2026-06-02 (Alembic 0015 + _compute_bullpen_workload + MLB-API ingest module + tests). MLB-API ingest run + workload rebuild PENDING.</t>
         </is>
       </c>
     </row>
@@ -23376,7 +23376,7 @@
       </c>
       <c r="H237" s="46" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Code-complete</t>
         </is>
       </c>
       <c r="I237" s="46" t="inlineStr">
@@ -23401,7 +23401,7 @@
       </c>
       <c r="M237" s="46" t="inlineStr">
         <is>
-          <t>Distribution-shifting; flag-gated. Filed 2026-06-01.</t>
+          <t>Code-complete 2026-06-02, gated SIM_MANAGER OFF (pitch-count bug fixed; fatigue/TTO/reliever scoring + wiring + tests; flag-off byte-identical, regression-green). Enable + &gt;=400-sim validation + golden-fixture regen PENDING.</t>
         </is>
       </c>
     </row>
@@ -23443,7 +23443,7 @@
       </c>
       <c r="H238" s="46" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Code-complete</t>
         </is>
       </c>
       <c r="I238" s="46" t="inlineStr">
@@ -23468,7 +23468,7 @@
       </c>
       <c r="M238" s="46" t="inlineStr">
         <is>
-          <t>Filed 2026-06-01.</t>
+          <t>Code-complete 2026-06-02 (provider closing-line branch + scripts/load_historical_odds.py + tests). Live backfill run (ODDS_API_KEY + network) PENDING.</t>
         </is>
       </c>
     </row>

</xml_diff>